<commit_message>
Updates to account for the renaming of some code lists required by Form 2FC
</commit_message>
<xml_diff>
--- a/form_reporting_templates/Form-2FC.xlsx
+++ b/form_reporting_templates/Form-2FC.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28730"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\echassot\Desktop\repositories\data-reporting\iotc-reference-forms\form_reporting_templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFA97D32-F5F1-4904-9AE2-BB2B6C35EBAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFA12C53-3BD6-495D-BFA0-DC8FFDA898D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="wX8sA2MiVV4hem5/4RTiTmcDJYFB86HqbOVJt9hNWIZw6gEt8u041CW+Lo33VdE+XPx62lk39pDAbSFn1bENfA==" workbookSaltValue="4+KZsXogYyQ9Ht7v5WkMIg==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Metadata" sheetId="1" r:id="rId1"/>
@@ -2296,7 +2296,7 @@
       <c r="L55" s="36"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="kiQTEPL4oEo/2qZDsNw9GXsxKzjVlPg4a6Nc1pevXYFCxYI5O1RW1QMnQ7wJl2NCmbJbsu9xC5UCAm9KWirCqQ==" saltValue="4e6mAyh86NxjRxNgc0n2pw==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="5oUdzMZs4v1G3py9w2Jz0pbh87l+ggnYAgHBsNXeOnXee8TGb5Am7cFPTZr1wp5WPgYjICRheQiH0FgPo3Ye8A==" saltValue="624Zce3ETBd7WyhAZMcg8g==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
   <mergeCells count="6">
     <mergeCell ref="B2:O3"/>
     <mergeCell ref="C4:E4"/>
@@ -2323,11 +2323,11 @@
     <hyperlink ref="D5" r:id="rId2" location="sourcesFC" xr:uid="{D508B0C5-71F1-4418-BA5D-6D532A3A0D47}"/>
     <hyperlink ref="E5" r:id="rId3" location="processingsFC" xr:uid="{3B28F9E8-FD32-4256-82C2-97BF03FEE964}"/>
     <hyperlink ref="F5" r:id="rId4" location="coverageTypes" xr:uid="{15A256B6-6B98-4ABF-81CC-D96AC29A08E2}"/>
-    <hyperlink ref="H5" r:id="rId5" location="boatTypes" display="Type" xr:uid="{DADB17F2-537E-4DBC-AFEA-6EE304F8C6D0}"/>
+    <hyperlink ref="H5" r:id="rId5" location="vesselArchitectures" xr:uid="{DADB17F2-537E-4DBC-AFEA-6EE304F8C6D0}"/>
     <hyperlink ref="I5" r:id="rId6" location="mechanizationTypes" xr:uid="{40C3FFA1-CD46-4638-8E84-B19E43E165D4}"/>
     <hyperlink ref="J5" r:id="rId7" location="fishPreservationMethods" xr:uid="{2A56DBD0-E939-42A6-98DA-87DA852FD2E9}"/>
     <hyperlink ref="K5" r:id="rId8" location="fishStorageTypes" xr:uid="{9C5A0F26-DE48-4B7A-BF87-82196056DE69}"/>
-    <hyperlink ref="L5" r:id="rId9" location="boatClassTypes" xr:uid="{263265AE-A782-4C7E-A95B-56C7C8AA2144}"/>
+    <hyperlink ref="L5" r:id="rId9" location="vesselSizeTypes" xr:uid="{263265AE-A782-4C7E-A95B-56C7C8AA2144}"/>
     <hyperlink ref="B5" r:id="rId10" location="Vessel_Types" xr:uid="{9938127B-C147-49BE-9C85-EBE93EF4251D}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Update of form 2FC in link with the renaming of code list "Vessel architecture"
</commit_message>
<xml_diff>
--- a/form_reporting_templates/Form-2FC.xlsx
+++ b/form_reporting_templates/Form-2FC.xlsx
@@ -8,10 +8,10 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\echassot\Desktop\repositories\data-reporting\iotc-reference-forms\form_reporting_templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFA12C53-3BD6-495D-BFA0-DC8FFDA898D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F984D15-C229-4E54-BE88-038CD80F1EA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="wX8sA2MiVV4hem5/4RTiTmcDJYFB86HqbOVJt9hNWIZw6gEt8u041CW+Lo33VdE+XPx62lk39pDAbSFn1bENfA==" workbookSaltValue="4+KZsXogYyQ9Ht7v5WkMIg==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Metadata" sheetId="1" r:id="rId1"/>
@@ -81,9 +81,6 @@
     <t>Source coverage</t>
   </si>
   <si>
-    <t>Boat</t>
-  </si>
-  <si>
     <t>Mechanisation</t>
   </si>
   <si>
@@ -150,7 +147,10 @@
     <t>Vessel type</t>
   </si>
   <si>
-    <t>Configuration</t>
+    <t>Architecture</t>
+  </si>
+  <si>
+    <t>Vessel</t>
   </si>
 </sst>
 </file>
@@ -1207,7 +1207,7 @@
     <row r="1" spans="2:8" ht="7.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="68" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C2" s="69"/>
       <c r="D2" s="69"/>
@@ -1231,14 +1231,14 @@
         <v>9</v>
       </c>
       <c r="D4" s="15" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E4" s="16"/>
       <c r="F4" s="14" t="s">
         <v>7</v>
       </c>
       <c r="G4" s="17" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="H4" s="18"/>
     </row>
@@ -1274,12 +1274,12 @@
     <row r="8" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B8" s="19"/>
       <c r="C8" s="67" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D8" s="67"/>
       <c r="E8" s="20"/>
       <c r="F8" s="67" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G8" s="67"/>
       <c r="H8" s="21"/>
@@ -1300,12 +1300,12 @@
     <row r="10" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B10" s="19"/>
       <c r="C10" s="24" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D10" s="3"/>
       <c r="E10" s="20"/>
       <c r="F10" s="20" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G10" s="3"/>
       <c r="H10" s="21"/>
@@ -1322,7 +1322,7 @@
     <row r="12" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B12" s="19"/>
       <c r="C12" s="24" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D12" s="63"/>
       <c r="E12" s="20"/>
@@ -1393,7 +1393,7 @@
     <row r="19" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B19" s="19"/>
       <c r="C19" s="40" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D19" s="9"/>
       <c r="E19" s="20"/>
@@ -1404,7 +1404,7 @@
     <row r="20" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B20" s="19"/>
       <c r="C20" s="41" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D20" s="9"/>
       <c r="E20" s="20"/>
@@ -1513,7 +1513,7 @@
     <col min="12" max="12" width="9.140625" style="38"/>
     <col min="13" max="13" width="9.140625" style="48"/>
     <col min="14" max="14" width="9.140625" style="49"/>
-    <col min="15" max="15" width="9.140625" style="51"/>
+    <col min="15" max="15" width="10.5703125" style="51" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="7.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -1534,7 +1534,7 @@
     </row>
     <row r="2" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="68" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C2" s="69"/>
       <c r="D2" s="69"/>
@@ -1570,7 +1570,7 @@
     <row r="4" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4"/>
       <c r="B4" s="62" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C4" s="74" t="s">
         <v>12</v>
@@ -1582,25 +1582,25 @@
       </c>
       <c r="G4" s="76"/>
       <c r="H4" s="74" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="I4" s="76"/>
       <c r="J4" s="74" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K4" s="76"/>
       <c r="L4" s="74" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M4" s="75"/>
       <c r="N4" s="76"/>
       <c r="O4" s="33" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="5" spans="1:15" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B5" s="55" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C5" s="61" t="s">
         <v>8</v>
@@ -1615,31 +1615,31 @@
         <v>8</v>
       </c>
       <c r="G5" s="53" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H5" s="55" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="I5" s="56" t="s">
+        <v>14</v>
+      </c>
+      <c r="J5" s="55" t="s">
         <v>15</v>
       </c>
-      <c r="J5" s="55" t="s">
-        <v>16</v>
-      </c>
       <c r="K5" s="56" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="L5" s="55" t="s">
         <v>8</v>
       </c>
       <c r="M5" s="59" t="s">
+        <v>18</v>
+      </c>
+      <c r="N5" s="60" t="s">
         <v>19</v>
       </c>
-      <c r="N5" s="60" t="s">
+      <c r="O5" s="54" t="s">
         <v>20</v>
-      </c>
-      <c r="O5" s="54" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
@@ -2296,7 +2296,8 @@
       <c r="L55" s="36"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="5oUdzMZs4v1G3py9w2Jz0pbh87l+ggnYAgHBsNXeOnXee8TGb5Am7cFPTZr1wp5WPgYjICRheQiH0FgPo3Ye8A==" saltValue="624Zce3ETBd7WyhAZMcg8g==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
+  <sheetProtection selectLockedCells="1"/>
+  <dataConsolidate/>
   <mergeCells count="6">
     <mergeCell ref="B2:O3"/>
     <mergeCell ref="C4:E4"/>
@@ -2323,7 +2324,7 @@
     <hyperlink ref="D5" r:id="rId2" location="sourcesFC" xr:uid="{D508B0C5-71F1-4418-BA5D-6D532A3A0D47}"/>
     <hyperlink ref="E5" r:id="rId3" location="processingsFC" xr:uid="{3B28F9E8-FD32-4256-82C2-97BF03FEE964}"/>
     <hyperlink ref="F5" r:id="rId4" location="coverageTypes" xr:uid="{15A256B6-6B98-4ABF-81CC-D96AC29A08E2}"/>
-    <hyperlink ref="H5" r:id="rId5" location="vesselArchitectures" xr:uid="{DADB17F2-537E-4DBC-AFEA-6EE304F8C6D0}"/>
+    <hyperlink ref="H5" r:id="rId5" location="vesselArchitectures" display="Configuration" xr:uid="{DADB17F2-537E-4DBC-AFEA-6EE304F8C6D0}"/>
     <hyperlink ref="I5" r:id="rId6" location="mechanizationTypes" xr:uid="{40C3FFA1-CD46-4638-8E84-B19E43E165D4}"/>
     <hyperlink ref="J5" r:id="rId7" location="fishPreservationMethods" xr:uid="{2A56DBD0-E939-42A6-98DA-87DA852FD2E9}"/>
     <hyperlink ref="K5" r:id="rId8" location="fishStorageTypes" xr:uid="{9C5A0F26-DE48-4B7A-BF87-82196056DE69}"/>

</xml_diff>

<commit_message>
Correction of URL for the architecture code list
</commit_message>
<xml_diff>
--- a/form_reporting_templates/Form-2FC.xlsx
+++ b/form_reporting_templates/Form-2FC.xlsx
@@ -1,17 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\echassot\Desktop\repositories\data-reporting\iotc-reference-forms\form_reporting_templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F984D15-C229-4E54-BE88-038CD80F1EA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="wX8sA2MiVV4hem5/4RTiTmcDJYFB86HqbOVJt9hNWIZw6gEt8u041CW+Lo33VdE+XPx62lk39pDAbSFn1bENfA==" workbookSaltValue="4+KZsXogYyQ9Ht7v5WkMIg==" workbookSpinCount="100000" lockStructure="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E818B382-EE7F-4062-9B7B-F8F581A6D419}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Metadata" sheetId="1" r:id="rId1"/>
@@ -1508,7 +1507,7 @@
     <col min="7" max="7" width="11.42578125" style="45" customWidth="1"/>
     <col min="8" max="8" width="15.7109375" style="38" customWidth="1"/>
     <col min="9" max="9" width="14.28515625" style="39" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.140625" style="38" customWidth="1"/>
+    <col min="10" max="10" width="14" style="38" customWidth="1"/>
     <col min="11" max="11" width="12.140625" style="39" customWidth="1"/>
     <col min="12" max="12" width="9.140625" style="38"/>
     <col min="13" max="13" width="9.140625" style="48"/>
@@ -2296,7 +2295,7 @@
       <c r="L55" s="36"/>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="T2FNfLpWoT4MRg2otK51La72TU7anAWdRVRKvX4TcPEZkqT6m5RJdYYIE81yBloSvx9azOJ1luGQeY9oKxHqzg==" saltValue="1DTaXmGskjbnUEofOKc/lg==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <dataConsolidate/>
   <mergeCells count="6">
     <mergeCell ref="B2:O3"/>
@@ -2324,7 +2323,7 @@
     <hyperlink ref="D5" r:id="rId2" location="sourcesFC" xr:uid="{D508B0C5-71F1-4418-BA5D-6D532A3A0D47}"/>
     <hyperlink ref="E5" r:id="rId3" location="processingsFC" xr:uid="{3B28F9E8-FD32-4256-82C2-97BF03FEE964}"/>
     <hyperlink ref="F5" r:id="rId4" location="coverageTypes" xr:uid="{15A256B6-6B98-4ABF-81CC-D96AC29A08E2}"/>
-    <hyperlink ref="H5" r:id="rId5" location="vesselArchitectures" display="Configuration" xr:uid="{DADB17F2-537E-4DBC-AFEA-6EE304F8C6D0}"/>
+    <hyperlink ref="H5" r:id="rId5" location="Vessel_Architectures" xr:uid="{DADB17F2-537E-4DBC-AFEA-6EE304F8C6D0}"/>
     <hyperlink ref="I5" r:id="rId6" location="mechanizationTypes" xr:uid="{40C3FFA1-CD46-4638-8E84-B19E43E165D4}"/>
     <hyperlink ref="J5" r:id="rId7" location="fishPreservationMethods" xr:uid="{2A56DBD0-E939-42A6-98DA-87DA852FD2E9}"/>
     <hyperlink ref="K5" r:id="rId8" location="fishStorageTypes" xr:uid="{9C5A0F26-DE48-4B7A-BF87-82196056DE69}"/>

</xml_diff>

<commit_message>
update of name and url of vessel measurement types in 2FC form
</commit_message>
<xml_diff>
--- a/form_reporting_templates/Form-2FC.xlsx
+++ b/form_reporting_templates/Form-2FC.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\echassot\Desktop\repositories\data-reporting\iotc-reference-forms\form_reporting_templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E818B382-EE7F-4062-9B7B-F8F581A6D419}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D10AD1F-0D59-4409-8F1A-67AE9B3AE846}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Metadata" sheetId="1" r:id="rId1"/>
@@ -1472,7 +1472,7 @@
       <c r="D27" s="2"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="KNUMqZKJ4N+zQSICBOfly4QIN4w7uPj7XhnHLy59nurDreAcWdF/itYUewjYLJ+XVsqgPlni/onwMcqlC+01uw==" saltValue="xXKb0qXqoHvpEa2Suso0Kw==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="+4pTJJ3lVm1rc8SJ6itnkxBD6VLH/wnTJwlZMG/wA+B3ITInRxnXH9qtCb1Lk9puVgUylUC9seGZW9ea0SthcA==" saltValue="FOemv+3C2Z3iBrzoYAeBBw==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
   <mergeCells count="4">
     <mergeCell ref="C25:G25"/>
     <mergeCell ref="C8:D8"/>
@@ -1486,7 +1486,7 @@
   </dataValidations>
   <hyperlinks>
     <hyperlink ref="C19" r:id="rId1" location="entities" xr:uid="{1442B3F2-6122-44BA-A4A6-8B72CAE14165}"/>
-    <hyperlink ref="C20" r:id="rId2" location="countries" display="Flag country" xr:uid="{36E4CE57-0E51-4624-84D7-B89CC49ED5B7}"/>
+    <hyperlink ref="C20" r:id="rId2" location="countries" xr:uid="{36E4CE57-0E51-4624-84D7-B89CC49ED5B7}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>
@@ -2295,7 +2295,7 @@
       <c r="L55" s="36"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="T2FNfLpWoT4MRg2otK51La72TU7anAWdRVRKvX4TcPEZkqT6m5RJdYYIE81yBloSvx9azOJ1luGQeY9oKxHqzg==" saltValue="1DTaXmGskjbnUEofOKc/lg==" spinCount="100000" sheet="1" selectLockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="4ySVKZctl9irT+AViY1Wya3Wh5ym6rvESMIBhN0W412WOIYCnFKP2S7gsjcBT+UVNJr4qeoFgGtS0kNMBYeCkA==" saltValue="w6RnUiOPMdJKDIvuDCQlVA==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <dataConsolidate/>
   <mergeCells count="6">
     <mergeCell ref="B2:O3"/>
@@ -2327,7 +2327,7 @@
     <hyperlink ref="I5" r:id="rId6" location="mechanizationTypes" xr:uid="{40C3FFA1-CD46-4638-8E84-B19E43E165D4}"/>
     <hyperlink ref="J5" r:id="rId7" location="fishPreservationMethods" xr:uid="{2A56DBD0-E939-42A6-98DA-87DA852FD2E9}"/>
     <hyperlink ref="K5" r:id="rId8" location="fishStorageTypes" xr:uid="{9C5A0F26-DE48-4B7A-BF87-82196056DE69}"/>
-    <hyperlink ref="L5" r:id="rId9" location="vesselSizeTypes" xr:uid="{263265AE-A782-4C7E-A95B-56C7C8AA2144}"/>
+    <hyperlink ref="L5" r:id="rId9" location="Vessel_Measurement_Types" xr:uid="{263265AE-A782-4C7E-A95B-56C7C8AA2144}"/>
     <hyperlink ref="B5" r:id="rId10" location="Vessel_Types" xr:uid="{9938127B-C147-49BE-9C85-EBE93EF4251D}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>